<commit_message>
Integra Maps, roteiro por distancia e ficha de anamnese no app.
Links Google Maps no inventario e PDF do roteiro; ordem das visitas otimizada por dia; geracao de fichas medicas na aba 4 (desktop e Streamlit).

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/Modelo_Inventario_Turistico.xlsx
+++ b/data/Modelo_Inventario_Turistico.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USI-SEVEN\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USI-SEVEN\OneDrive\Desktop\PROJETO INTEGRADOR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5570C12-7FB3-4820-8043-45BBFCBDCC4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75171219-9E42-4E44-B800-2A76B6E73EA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="128">
   <si>
     <t>ID</t>
   </si>
@@ -209,9 +209,6 @@
     <t>Hospedagem / Ecoturismo</t>
   </si>
   <si>
-    <t>Sítio Tainã — Hospedagem e Natureza</t>
-  </si>
-  <si>
     <t>Hospedagem rural associada ao descanso e contato com a natureza; referências a trilhas/camping em materiais antigos precisam ser verificadas.</t>
   </si>
   <si>
@@ -282,13 +279,139 @@
   </si>
   <si>
     <t>ART_21</t>
+  </si>
+  <si>
+    <t>Pinacoteca Fórum das Artes</t>
+  </si>
+  <si>
+    <t>Cultura</t>
+  </si>
+  <si>
+    <t>Museu em prédio histórico, ambiente fechado, seguro e roteiro estruturado.</t>
+  </si>
+  <si>
+    <t>Catedral Metropolitana de Sant'Ana</t>
+  </si>
+  <si>
+    <t>Atração central, fácil acesso, ideal para turistas comodistas.</t>
+  </si>
+  <si>
+    <t>Trilha com degraus estruturados, exige disposição física moderada e contato com a mata.</t>
+  </si>
+  <si>
+    <t>Base da Nuvem (Voo Livre)</t>
+  </si>
+  <si>
+    <t>Aventura alta (Plog alto), porém operada por profissionais e agências (Cohen baixo/médio).</t>
+  </si>
+  <si>
+    <t>ATR_22</t>
+  </si>
+  <si>
+    <t>ATR_23</t>
+  </si>
+  <si>
+    <t>ATR_24</t>
+  </si>
+  <si>
+    <t>ATR_25</t>
+  </si>
+  <si>
+    <t>Botucatu - SP</t>
+  </si>
+  <si>
+    <t>Maps</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/dfXSyxybbzTdReHU8</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/QFtCy2PmeuHxHjy17</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/Ts9GPJ9S4vbugAyt7</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/Y5q6Ti2JvnmMrqKEA</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/Gm6JtXThEY7kgbJZA</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/22wx6ECWQFEFtRMX8</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/NN2h77d5ogcCRp45A</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/rvfL7sjp9buWsQ63A</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/wE4htaFRTrZhXCUz9</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/ghR8Jr6htaRTaHGz8</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/3A3zcFWB3tiYTEUXA</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/z5hZYborYAWAmPCM9</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/LLNyu2byWzJZd5729</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/tCzY9n5U8L1wCae99</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/TDghVrB2mJoqpLC36</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/hqBDUZ7znecFDJDWA</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/e7JQA75weJy5wD6P6</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/TrjFoEriA3iZFopr5</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/kSb3B3eyqKsoBDUK8</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/vDzB9RRj6x1oJepx9</t>
+  </si>
+  <si>
+    <t>Sítio Tainã</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/YytCaytK3NPEX4oo8</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/qi7odsf4qjbQGXmq6</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/ErxLMDTmDZx5p3tq6</t>
+  </si>
+  <si>
+    <t>Parque Natural Municipal Cachoeira da Marta</t>
+  </si>
+  <si>
+    <t>Ecoturismo</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/FzQcFhBJnbY9DV2K7</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/Be2otkH5CXmaaL5F7</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -311,6 +434,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -349,7 +480,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -377,42 +508,103 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFA6A6A6"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFA6A6A6"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFA6A6A6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFA6A6A6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="46" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="46" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="15">
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -426,20 +618,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="InventarioTuristico" displayName="InventarioTuristico" ref="A1:K2" insertRow="1">
-  <autoFilter ref="A1:K2" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Nome da Atração"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Categoria"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Horário de Abertura"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Horário de Fechamento"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Capacidade Máx. Grupo (Pessoas)"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Tempo Médio (horas)"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Peso Plog (Aventura)"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Peso Cohen (Independência)"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Descrição Breve"/>
-    <tableColumn id="11" xr3:uid="{A35E046A-1AE6-47DD-8906-B085D349D97F}" name="Cidade"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="InventarioTuristico" displayName="InventarioTuristico" ref="A1:L2" insertRow="1" headerRowDxfId="14" dataDxfId="13" totalsRowDxfId="12">
+  <autoFilter ref="A1:L2" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Nome da Atração" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Categoria" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Horário de Abertura" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Horário de Fechamento" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Capacidade Máx. Grupo (Pessoas)" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Tempo Médio (horas)" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Peso Plog (Aventura)" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Peso Cohen (Independência)" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Descrição Breve" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{A35E046A-1AE6-47DD-8906-B085D349D97F}" name="Cidade" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{5A74869C-D614-4A67-B17E-B49AC67DB5EA}" name="Maps" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -730,76 +923,80 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.5546875" customWidth="1"/>
     <col min="4" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="16" customWidth="1"/>
-    <col min="10" max="10" width="86.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="86.33203125" customWidth="1"/>
     <col min="11" max="11" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="40.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="7" t="s">
         <v>9</v>
       </c>
       <c r="K1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="5"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-    </row>
-    <row r="3" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+        <v>63</v>
+      </c>
+      <c r="L1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="2"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+    </row>
+    <row r="3" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="12">
+      <c r="D3" s="4">
         <v>0.33333333333333331</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="4">
         <v>0.70833333333333337</v>
       </c>
       <c r="F3">
@@ -814,34 +1011,37 @@
       <c r="I3">
         <v>3</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="J3" s="10" t="s">
         <v>17</v>
       </c>
       <c r="K3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="L3" s="13" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B4" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" s="10" t="s">
         <v>18</v>
       </c>
       <c r="C4" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="12">
+      <c r="D4" s="4">
         <v>0.33333333333333331</v>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="4">
         <v>0.70833333333333337</v>
       </c>
       <c r="F4">
         <v>20</v>
       </c>
       <c r="G4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -849,34 +1049,37 @@
       <c r="I4">
         <v>2</v>
       </c>
-      <c r="J4" s="8" t="s">
+      <c r="J4" s="10" t="s">
         <v>20</v>
       </c>
       <c r="K4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="L4" s="13" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>68</v>
-      </c>
-      <c r="B5" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" s="10" t="s">
         <v>21</v>
       </c>
       <c r="C5" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="12">
+      <c r="D5" s="4">
         <v>0.375</v>
       </c>
-      <c r="E5" s="12">
+      <c r="E5" s="4">
         <v>0.70833333333333337</v>
       </c>
       <c r="F5">
         <v>15</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H5">
         <v>1</v>
@@ -884,34 +1087,37 @@
       <c r="I5">
         <v>2</v>
       </c>
-      <c r="J5" s="8" t="s">
+      <c r="J5" s="10" t="s">
         <v>22</v>
       </c>
       <c r="K5" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="L5" s="13" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>69</v>
-      </c>
-      <c r="B6" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>23</v>
       </c>
       <c r="C6" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="12">
+      <c r="D6" s="4">
         <v>0.45833333333333331</v>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="4">
         <v>0.75</v>
       </c>
       <c r="F6">
         <v>10</v>
       </c>
       <c r="G6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H6">
         <v>4</v>
@@ -919,27 +1125,30 @@
       <c r="I6">
         <v>3</v>
       </c>
-      <c r="J6" s="8" t="s">
+      <c r="J6" s="10" t="s">
         <v>24</v>
       </c>
       <c r="K6" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="L6" s="13" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>70</v>
-      </c>
-      <c r="B7" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="4">
         <v>0.41666666666666669</v>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="4">
         <v>0.66666666666666663</v>
       </c>
       <c r="F7">
@@ -954,34 +1163,37 @@
       <c r="I7">
         <v>3</v>
       </c>
-      <c r="J7" s="8" t="s">
+      <c r="J7" s="10" t="s">
         <v>27</v>
       </c>
       <c r="K7" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="L7" s="13" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>71</v>
-      </c>
-      <c r="B8" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="12">
+      <c r="D8" s="4">
         <v>0.375</v>
       </c>
-      <c r="E8" s="12">
+      <c r="E8" s="4">
         <v>0.70833333333333337</v>
       </c>
       <c r="F8">
         <v>15</v>
       </c>
       <c r="G8">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="H8">
         <v>2</v>
@@ -989,27 +1201,30 @@
       <c r="I8">
         <v>4</v>
       </c>
-      <c r="J8" s="8" t="s">
+      <c r="J8" s="10" t="s">
         <v>29</v>
       </c>
       <c r="K8" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="L8" s="13" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>72</v>
-      </c>
-      <c r="B9" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B9" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="4">
         <v>0.375</v>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="4">
         <v>0.75</v>
       </c>
       <c r="F9">
@@ -1024,27 +1239,30 @@
       <c r="I9">
         <v>4</v>
       </c>
-      <c r="J9" s="8" t="s">
+      <c r="J9" s="10" t="s">
         <v>31</v>
       </c>
       <c r="K9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="L9" s="13" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>73</v>
-      </c>
-      <c r="B10" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" t="s">
         <v>33</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="4">
         <v>0.375</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="4">
         <v>0.66666666666666663</v>
       </c>
       <c r="F10">
@@ -1059,27 +1277,30 @@
       <c r="I10">
         <v>2</v>
       </c>
-      <c r="J10" s="8" t="s">
+      <c r="J10" s="10" t="s">
         <v>34</v>
       </c>
       <c r="K10" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="L10" s="13" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="12">
+      <c r="D11" s="4">
         <v>0.41666666666666669</v>
       </c>
-      <c r="E11" s="12">
+      <c r="E11" s="4">
         <v>0.70833333333333337</v>
       </c>
       <c r="F11">
@@ -1094,27 +1315,30 @@
       <c r="I11">
         <v>5</v>
       </c>
-      <c r="J11" s="8" t="s">
+      <c r="J11" s="10" t="s">
         <v>36</v>
       </c>
       <c r="K11" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="L11" s="13" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>75</v>
-      </c>
-      <c r="B12" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B12" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="12">
+      <c r="D12" s="4">
         <v>0.33333333333333331</v>
       </c>
-      <c r="E12" s="12">
+      <c r="E12" s="4">
         <v>0.75</v>
       </c>
       <c r="F12">
@@ -1129,27 +1353,30 @@
       <c r="I12">
         <v>4</v>
       </c>
-      <c r="J12" s="8" t="s">
+      <c r="J12" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K12" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="L12" s="13" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>76</v>
-      </c>
-      <c r="B13" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B13" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" t="s">
         <v>40</v>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="4">
         <v>0.47916666666666669</v>
       </c>
-      <c r="E13" s="12">
+      <c r="E13" s="4">
         <v>0.58333333333333337</v>
       </c>
       <c r="F13">
@@ -1164,27 +1391,30 @@
       <c r="I13">
         <v>4</v>
       </c>
-      <c r="J13" s="8" t="s">
+      <c r="J13" s="10" t="s">
         <v>41</v>
       </c>
       <c r="K13" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="L13" s="13" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>77</v>
-      </c>
-      <c r="B14" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B14" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" t="s">
         <v>40</v>
       </c>
-      <c r="D14" s="12">
+      <c r="D14" s="4">
         <v>0.47916666666666669</v>
       </c>
-      <c r="E14" s="12">
+      <c r="E14" s="4">
         <v>0.58333333333333337</v>
       </c>
       <c r="F14">
@@ -1199,27 +1429,30 @@
       <c r="I14">
         <v>2</v>
       </c>
-      <c r="J14" s="8" t="s">
+      <c r="J14" s="10" t="s">
         <v>43</v>
       </c>
       <c r="K14" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="L14" s="13" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>78</v>
-      </c>
-      <c r="B15" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B15" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" t="s">
         <v>40</v>
       </c>
-      <c r="D15" s="12">
+      <c r="D15" s="4">
         <v>0.33333333333333331</v>
       </c>
-      <c r="E15" s="12">
+      <c r="E15" s="4">
         <v>0.70833333333333337</v>
       </c>
       <c r="F15">
@@ -1229,32 +1462,35 @@
         <v>1</v>
       </c>
       <c r="H15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I15">
         <v>3</v>
       </c>
-      <c r="J15" s="8" t="s">
+      <c r="J15" s="10" t="s">
         <v>45</v>
       </c>
       <c r="K15" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="L15" s="13" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>79</v>
-      </c>
-      <c r="B16" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B16" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" t="s">
         <v>40</v>
       </c>
-      <c r="D16" s="12">
+      <c r="D16" s="4">
         <v>0.45833333333333331</v>
       </c>
-      <c r="E16" s="12">
+      <c r="E16" s="4">
         <v>0.625</v>
       </c>
       <c r="F16">
@@ -1264,102 +1500,111 @@
         <v>2</v>
       </c>
       <c r="H16">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I16">
         <v>3</v>
       </c>
-      <c r="J16" s="8" t="s">
+      <c r="J16" s="10" t="s">
         <v>47</v>
       </c>
       <c r="K16" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="L16" s="13" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>80</v>
-      </c>
-      <c r="B17" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="B17" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" t="s">
         <v>40</v>
       </c>
-      <c r="D17" s="12">
+      <c r="D17" s="4">
         <v>0.45833333333333331</v>
       </c>
-      <c r="E17" s="12">
+      <c r="E17" s="4">
         <v>0.60416666666666663</v>
       </c>
       <c r="F17">
         <v>20</v>
       </c>
       <c r="G17">
+        <v>1.5</v>
+      </c>
+      <c r="H17">
         <v>2</v>
-      </c>
-      <c r="H17">
-        <v>1</v>
       </c>
       <c r="I17">
         <v>4</v>
       </c>
-      <c r="J17" s="8" t="s">
+      <c r="J17" s="10" t="s">
         <v>49</v>
       </c>
       <c r="K17" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="L17" s="13" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>81</v>
-      </c>
-      <c r="B18" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="B18" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" t="s">
         <v>40</v>
       </c>
-      <c r="D18" s="12">
+      <c r="D18" s="4">
         <v>0.41666666666666669</v>
       </c>
-      <c r="E18" s="12">
+      <c r="E18" s="4">
         <v>0.75</v>
       </c>
       <c r="F18">
         <v>15</v>
       </c>
       <c r="G18">
+        <v>1</v>
+      </c>
+      <c r="H18">
         <v>2</v>
-      </c>
-      <c r="H18">
-        <v>1</v>
       </c>
       <c r="I18">
         <v>5</v>
       </c>
-      <c r="J18" s="8" t="s">
+      <c r="J18" s="10" t="s">
         <v>51</v>
       </c>
       <c r="K18" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="L18" s="13" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>82</v>
-      </c>
-      <c r="B19" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="B19" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" t="s">
         <v>53</v>
       </c>
-      <c r="D19" s="12">
+      <c r="D19" s="4">
         <v>0</v>
       </c>
-      <c r="E19" s="13">
+      <c r="E19" s="6">
         <v>1</v>
       </c>
       <c r="F19">
@@ -1371,27 +1616,30 @@
       <c r="I19">
         <v>5</v>
       </c>
-      <c r="J19" s="8" t="s">
+      <c r="J19" s="10" t="s">
         <v>54</v>
       </c>
       <c r="K19" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="L19" s="13" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>83</v>
-      </c>
-      <c r="B20" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B20" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" t="s">
         <v>53</v>
       </c>
-      <c r="D20" s="12">
+      <c r="D20" s="4">
         <v>0</v>
       </c>
-      <c r="E20" s="13">
+      <c r="E20" s="6">
         <v>1</v>
       </c>
       <c r="F20">
@@ -1403,34 +1651,37 @@
       <c r="I20">
         <v>3</v>
       </c>
-      <c r="J20" s="8" t="s">
+      <c r="J20" s="10" t="s">
         <v>56</v>
       </c>
       <c r="K20" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="L20" s="13" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>84</v>
-      </c>
-      <c r="B21" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="B21" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" t="s">
         <v>61</v>
       </c>
-      <c r="D21" s="12">
+      <c r="D21" s="4">
         <v>0</v>
       </c>
-      <c r="E21" s="13">
+      <c r="E21" s="6">
         <v>1</v>
       </c>
       <c r="F21">
         <v>15</v>
       </c>
       <c r="G21">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H21">
         <v>3</v>
@@ -1438,27 +1689,30 @@
       <c r="I21">
         <v>3</v>
       </c>
-      <c r="J21" s="8" t="s">
+      <c r="J21" s="10" t="s">
         <v>58</v>
       </c>
       <c r="K21" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="L21" s="13" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>85</v>
-      </c>
-      <c r="B22" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="B22" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C22" t="s">
         <v>53</v>
       </c>
-      <c r="D22" s="12">
+      <c r="D22" s="4">
         <v>0</v>
       </c>
-      <c r="E22" s="13">
+      <c r="E22" s="6">
         <v>1</v>
       </c>
       <c r="F22">
@@ -1470,27 +1724,30 @@
       <c r="I22">
         <v>1</v>
       </c>
-      <c r="J22" s="8" t="s">
+      <c r="J22" s="10" t="s">
         <v>60</v>
       </c>
       <c r="K22" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="L22" s="13" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>86</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="C23" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="C23" t="s">
         <v>53</v>
       </c>
-      <c r="D23" s="12">
+      <c r="D23" s="4">
         <v>0</v>
       </c>
-      <c r="E23" s="13">
+      <c r="E23" s="6">
         <v>1</v>
       </c>
       <c r="F23">
@@ -1502,23 +1759,182 @@
       <c r="I23">
         <v>4</v>
       </c>
-      <c r="J23" s="8" t="s">
-        <v>63</v>
+      <c r="J23" s="10" t="s">
+        <v>62</v>
       </c>
       <c r="K23" t="s">
-        <v>65</v>
+        <v>64</v>
+      </c>
+      <c r="L23" s="13" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>94</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="F24" s="12">
+        <v>50</v>
+      </c>
+      <c r="G24" s="12">
+        <v>1.5</v>
+      </c>
+      <c r="H24" s="12">
+        <v>1</v>
+      </c>
+      <c r="I24" s="12">
+        <v>1</v>
+      </c>
+      <c r="J24" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="K24" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="L24" s="13" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>95</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F25" s="12">
+        <v>100</v>
+      </c>
+      <c r="G25" s="12">
+        <v>1</v>
+      </c>
+      <c r="H25" s="12">
+        <v>1</v>
+      </c>
+      <c r="I25" s="12">
+        <v>1</v>
+      </c>
+      <c r="J25" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="K25" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="L25" s="13" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>96</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="F26" s="12">
+        <v>15</v>
+      </c>
+      <c r="G26" s="12">
+        <v>1</v>
+      </c>
+      <c r="H26" s="12">
+        <v>4</v>
+      </c>
+      <c r="I26" s="12">
+        <v>3</v>
+      </c>
+      <c r="J26" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="K26" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="L26" s="13" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>97</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F27" s="12">
+        <v>10</v>
+      </c>
+      <c r="G27" s="12">
+        <v>1</v>
+      </c>
+      <c r="H27" s="12">
+        <v>4</v>
+      </c>
+      <c r="I27" s="12">
+        <v>3</v>
+      </c>
+      <c r="J27" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="K27" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="L27" s="13" t="s">
+        <v>127</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" errorTitle="Peso inválido" error="Escolha um valor de 1 a 5 na lista." sqref="H2:I495" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" errorTitle="Peso inválido" error="Escolha um valor de 1 a 5 na lista." sqref="H2:I23 H28:I491" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="L3" r:id="rId1" xr:uid="{3A9E559C-E701-4298-9B32-C0F6A4C09D36}"/>
+    <hyperlink ref="L4" r:id="rId2" xr:uid="{35DA58B3-0EEF-4264-B29D-FD45C76B46F6}"/>
+    <hyperlink ref="L5" r:id="rId3" xr:uid="{10356EE8-07AF-42AB-9DD3-4E860BE28A1D}"/>
+    <hyperlink ref="L6" r:id="rId4" xr:uid="{228C2F61-E5AC-4234-9808-1896811C3DCB}"/>
+    <hyperlink ref="L7" r:id="rId5" xr:uid="{FC9BBC5F-00DE-4114-9A78-7000EF3C4C2E}"/>
+    <hyperlink ref="L8" r:id="rId6" xr:uid="{DDA62292-96F3-448B-9030-36F9276C5AC8}"/>
+    <hyperlink ref="L9" r:id="rId7" xr:uid="{AC6ACB57-E02C-45CB-B4F9-168FF7ED3AA4}"/>
+    <hyperlink ref="L10" r:id="rId8" xr:uid="{94DB2CFE-932B-441D-ABFF-CC2514F23539}"/>
+    <hyperlink ref="L11" r:id="rId9" xr:uid="{506E84A3-CBB1-48A0-9F30-3A2BBEE8929A}"/>
+    <hyperlink ref="L12" r:id="rId10" xr:uid="{40665473-C667-41DA-A20C-8322113838ED}"/>
+    <hyperlink ref="L13" r:id="rId11" xr:uid="{5FA195CB-44C3-486F-94FF-5B8B0A610E33}"/>
+    <hyperlink ref="L14" r:id="rId12" xr:uid="{6FA33AD2-FA14-4748-ADE0-4C43ECBF7F3E}"/>
+    <hyperlink ref="L15" r:id="rId13" xr:uid="{9F474316-C92D-4019-8595-92EE5E655FF6}"/>
+    <hyperlink ref="L16" r:id="rId14" xr:uid="{FD5526D1-0CF1-486B-B275-ECA9AF1D0DCC}"/>
+    <hyperlink ref="L17" r:id="rId15" xr:uid="{0CE69685-C3DC-4DEA-893A-69C00C7F3701}"/>
+    <hyperlink ref="L18" r:id="rId16" xr:uid="{7D7AC133-60D5-4D28-8054-58DA677B893B}"/>
+    <hyperlink ref="L19" r:id="rId17" xr:uid="{21479737-5F4F-486C-8F53-13C64A08D7CA}"/>
+    <hyperlink ref="L21" r:id="rId18" xr:uid="{457B970B-FC58-4EBA-8112-1F20DA8E96F8}"/>
+    <hyperlink ref="L20" r:id="rId19" xr:uid="{E71BD71C-A5A6-45DC-BBAB-54103D918235}"/>
+    <hyperlink ref="L22" r:id="rId20" xr:uid="{25590415-0887-4B16-9CA5-EE871A05278E}"/>
+    <hyperlink ref="L23" r:id="rId21" xr:uid="{7E1AB2AB-AEEC-4AA5-99D2-0CF5A0626450}"/>
+    <hyperlink ref="L24" r:id="rId22" xr:uid="{D25139C7-1340-4017-958A-4F5FD286BDF5}"/>
+    <hyperlink ref="L25" r:id="rId23" xr:uid="{494EE29E-8499-41A8-B7D0-1E1FD7E1D14A}"/>
+    <hyperlink ref="L26" r:id="rId24" xr:uid="{69E9B54B-DF12-4D4A-B22B-2160B4E6353D}"/>
+    <hyperlink ref="L27" r:id="rId25" xr:uid="{79C7B52E-6CF6-4770-9FA7-9CF9775B579A}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId26"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId27"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>